<commit_message>
Publicar 84 ejemplares verificados y disponibles
</commit_message>
<xml_diff>
--- a/evento/Operacion_Evento_Trueque_IUB_2026-10-30.xlsx
+++ b/evento/Operacion_Evento_Trueque_IUB_2026-10-30.xlsx
@@ -8010,10 +8010,14 @@
           <t>Johana Brewne Kelly</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr"/>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E2" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F2" s="9" t="inlineStr"/>
@@ -8037,10 +8041,14 @@
           <t>Kelly Johana Brewne</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr"/>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr"/>
@@ -8064,10 +8072,14 @@
           <t>Michael Blake</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr"/>
@@ -8091,10 +8103,14 @@
           <t>Gerardo Meneses</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr"/>
@@ -8118,10 +8134,14 @@
           <t>John Green</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr"/>
@@ -8145,10 +8165,14 @@
           <t>Flor Salvador</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr"/>
@@ -8172,10 +8196,14 @@
           <t>Luis Maria Pescetti</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr"/>
@@ -8199,10 +8227,14 @@
           <t>Jose Manuel Grima, Alicia le Fur</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr"/>
@@ -8226,10 +8258,14 @@
           <t>Gabriel Garcia Marquez</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr"/>
@@ -8253,10 +8289,14 @@
           <t>Perret Gentil Beatriz</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr"/>
@@ -8280,10 +8320,14 @@
           <t>Beatriz Perret Gentil</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr"/>
@@ -8307,10 +8351,14 @@
           <t>Neale Donald</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr"/>
@@ -8334,10 +8382,14 @@
           <t>Gabriel Garcia Marquez</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr"/>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr"/>
@@ -8361,10 +8413,14 @@
           <t>Heredia Maria F.</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr"/>
@@ -8388,10 +8444,14 @@
           <t>Maria T. Balogh</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr"/>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr"/>
@@ -8415,10 +8475,14 @@
           <t>Maria T. Balogh</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr"/>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr"/>
@@ -8442,10 +8506,14 @@
           <t>Barreira Maria Arturo</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr"/>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr"/>
@@ -8469,10 +8537,14 @@
           <t>Arturo Barreira Maria</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr"/>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr"/>
@@ -8496,10 +8568,14 @@
           <t>Camilo Romero</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr"/>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr"/>
@@ -8523,10 +8599,14 @@
           <t>Flor Salvador</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr"/>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr"/>
@@ -8550,10 +8630,14 @@
           <t>Agatha Christie</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr"/>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr"/>
@@ -8577,10 +8661,14 @@
           <t>Bojunga Lygia</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr"/>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr"/>
@@ -8604,10 +8692,14 @@
           <t>Paulo Coelho</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr"/>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr"/>
@@ -8631,10 +8723,14 @@
           <t>Jorge Bucay</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr"/>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr"/>
@@ -8658,10 +8754,14 @@
           <t>Pedro Conrado Cudriz</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr"/>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr"/>
@@ -8685,10 +8785,14 @@
           <t>Osorio Lizarazo</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr"/>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr"/>
@@ -8712,10 +8816,14 @@
           <t>Robert Louis Stevenson</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr"/>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F28" s="9" t="inlineStr"/>
@@ -8739,10 +8847,14 @@
           <t>Stevenson</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr"/>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr"/>
@@ -8766,10 +8878,14 @@
           <t>Jorge Bustos</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr"/>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr"/>
@@ -8793,10 +8909,14 @@
           <t>Rhei Sofía</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr"/>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F31" s="9" t="inlineStr"/>
@@ -8820,10 +8940,14 @@
           <t>Juan Rulfo</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr"/>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F32" s="9" t="inlineStr"/>
@@ -8847,10 +8971,14 @@
           <t>Christine NÖstlinger</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr"/>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr"/>
@@ -8874,10 +9002,14 @@
           <t>Paulo Coelho</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr"/>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F34" s="9" t="inlineStr"/>
@@ -8901,10 +9033,14 @@
           <t>Celia Corral Cañas</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr"/>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr"/>
@@ -8928,10 +9064,14 @@
           <t>Angel Esteban, Stephanie Panichelli</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr"/>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E36" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr"/>
@@ -8955,10 +9095,14 @@
           <t>Paulina Aguilar Gutierrez</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr"/>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E37" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr"/>
@@ -8982,10 +9126,14 @@
           <t>Maria Cristina Ocampo de Manzano</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr"/>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr"/>
@@ -9009,10 +9157,14 @@
           <t>Ernesto Sabato</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr"/>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E39" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr"/>
@@ -9036,10 +9188,14 @@
           <t>Ernest Hemingway</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr"/>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E40" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr"/>
@@ -9063,10 +9219,14 @@
           <t>Castilla Julia M.</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr"/>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E41" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr"/>
@@ -9090,10 +9250,14 @@
           <t>Wayne Dyer</t>
         </is>
       </c>
-      <c r="D42" s="9" t="inlineStr"/>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E42" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr"/>
@@ -9117,10 +9281,14 @@
           <t>Elena Dreser</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr"/>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E43" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F43" s="9" t="inlineStr"/>
@@ -9144,10 +9312,14 @@
           <t>Maria Fernanda Heredia</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr"/>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F44" s="9" t="inlineStr"/>
@@ -9171,10 +9343,14 @@
           <t>James Clear</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr"/>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr"/>
@@ -9198,10 +9374,14 @@
           <t>Isabel Allende</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr"/>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr"/>
@@ -9225,10 +9405,14 @@
           <t>Marianamatilde Rodriguez Jaime</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr"/>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E47" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F47" s="9" t="inlineStr"/>
@@ -9252,10 +9436,14 @@
           <t>Alejandro Casona</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr"/>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E48" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F48" s="9" t="inlineStr"/>
@@ -9279,10 +9467,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr"/>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr"/>
@@ -9306,10 +9498,14 @@
           <t>Fernando de Rojas</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr"/>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F50" s="9" t="inlineStr"/>
@@ -9333,10 +9529,14 @@
           <t>Fernando de Rojas</t>
         </is>
       </c>
-      <c r="D51" s="9" t="inlineStr"/>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F51" s="9" t="inlineStr"/>
@@ -9360,10 +9560,14 @@
           <t>Adalberto Mieles Gómez</t>
         </is>
       </c>
-      <c r="D52" s="9" t="inlineStr"/>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F52" s="9" t="inlineStr"/>
@@ -9387,10 +9591,14 @@
           <t>Adalberto Mieles Gómez</t>
         </is>
       </c>
-      <c r="D53" s="9" t="inlineStr"/>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F53" s="9" t="inlineStr"/>
@@ -9414,10 +9622,14 @@
           <t>Jordi Sierra i Fabra</t>
         </is>
       </c>
-      <c r="D54" s="9" t="inlineStr"/>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F54" s="9" t="inlineStr"/>
@@ -9441,10 +9653,14 @@
           <t>Homero</t>
         </is>
       </c>
-      <c r="D55" s="9" t="inlineStr"/>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F55" s="9" t="inlineStr"/>
@@ -9468,10 +9684,14 @@
           <t>Zora Silvera Dany</t>
         </is>
       </c>
-      <c r="D56" s="9" t="inlineStr"/>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F56" s="9" t="inlineStr"/>
@@ -9495,10 +9715,14 @@
           <t>Dany Zora Silvera</t>
         </is>
       </c>
-      <c r="D57" s="9" t="inlineStr"/>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F57" s="9" t="inlineStr"/>
@@ -9522,10 +9746,14 @@
           <t>Arnoldo Palacios</t>
         </is>
       </c>
-      <c r="D58" s="9" t="inlineStr"/>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr"/>
@@ -9549,10 +9777,14 @@
           <t>Miguel de Cervantes Saavedra</t>
         </is>
       </c>
-      <c r="D59" s="9" t="inlineStr"/>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F59" s="9" t="inlineStr"/>
@@ -9576,10 +9808,14 @@
           <t>Miguel de Cervantes Saavedra</t>
         </is>
       </c>
-      <c r="D60" s="9" t="inlineStr"/>
+      <c r="D60" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F60" s="9" t="inlineStr"/>
@@ -9603,10 +9839,14 @@
           <t>Anonimo</t>
         </is>
       </c>
-      <c r="D61" s="9" t="inlineStr"/>
+      <c r="D61" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr"/>
@@ -9630,10 +9870,14 @@
           <t>Martin Orozco Cantillo</t>
         </is>
       </c>
-      <c r="D62" s="9" t="inlineStr"/>
+      <c r="D62" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F62" s="9" t="inlineStr"/>
@@ -9657,10 +9901,14 @@
           <t>Roumiguiére Cécile</t>
         </is>
       </c>
-      <c r="D63" s="9" t="inlineStr"/>
+      <c r="D63" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F63" s="9" t="inlineStr"/>
@@ -9684,10 +9932,14 @@
           <t>Corujo Elena</t>
         </is>
       </c>
-      <c r="D64" s="9" t="inlineStr"/>
+      <c r="D64" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F64" s="9" t="inlineStr"/>
@@ -9711,10 +9963,14 @@
           <t>Dalai Lama</t>
         </is>
       </c>
-      <c r="D65" s="9" t="inlineStr"/>
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F65" s="9" t="inlineStr"/>
@@ -9738,10 +9994,14 @@
           <t>Aguirre Sergio</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr"/>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F66" s="9" t="inlineStr"/>
@@ -9765,10 +10025,14 @@
           <t>Wade Davis</t>
         </is>
       </c>
-      <c r="D67" s="9" t="inlineStr"/>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F67" s="9" t="inlineStr"/>
@@ -9792,10 +10056,14 @@
           <t>Prieto Urina Carlos Daniel</t>
         </is>
       </c>
-      <c r="D68" s="9" t="inlineStr"/>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F68" s="9" t="inlineStr"/>
@@ -9819,10 +10087,14 @@
           <t>Carlos Daniel Prieto Urina</t>
         </is>
       </c>
-      <c r="D69" s="9" t="inlineStr"/>
+      <c r="D69" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F69" s="9" t="inlineStr"/>
@@ -9846,10 +10118,14 @@
           <t>Robin Norwood</t>
         </is>
       </c>
-      <c r="D70" s="9" t="inlineStr"/>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F70" s="9" t="inlineStr"/>
@@ -9873,10 +10149,14 @@
           <t>Gonzalo Maure Trenor</t>
         </is>
       </c>
-      <c r="D71" s="9" t="inlineStr"/>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F71" s="9" t="inlineStr"/>
@@ -9900,10 +10180,14 @@
           <t>Fiodor Dostoyevski</t>
         </is>
       </c>
-      <c r="D72" s="9" t="inlineStr"/>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F72" s="9" t="inlineStr"/>
@@ -9927,10 +10211,14 @@
           <t>Largion Barros de la Hoz</t>
         </is>
       </c>
-      <c r="D73" s="9" t="inlineStr"/>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F73" s="9" t="inlineStr"/>
@@ -9954,10 +10242,14 @@
           <t>Alvaro Miranda Villalobos</t>
         </is>
       </c>
-      <c r="D74" s="9" t="inlineStr"/>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F74" s="9" t="inlineStr"/>
@@ -9981,10 +10273,14 @@
           <t>Anonimo</t>
         </is>
       </c>
-      <c r="D75" s="9" t="inlineStr"/>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F75" s="9" t="inlineStr"/>
@@ -10008,10 +10304,14 @@
           <t>Mc Combie Karen</t>
         </is>
       </c>
-      <c r="D76" s="9" t="inlineStr"/>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F76" s="9" t="inlineStr"/>
@@ -10035,10 +10335,14 @@
           <t>Cristina Rebull</t>
         </is>
       </c>
-      <c r="D77" s="9" t="inlineStr"/>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F77" s="9" t="inlineStr"/>
@@ -10062,10 +10366,14 @@
           <t>Nostlinger Christine</t>
         </is>
       </c>
-      <c r="D78" s="9" t="inlineStr"/>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F78" s="9" t="inlineStr"/>
@@ -10089,10 +10397,14 @@
           <t>Flor Salvador</t>
         </is>
       </c>
-      <c r="D79" s="9" t="inlineStr"/>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F79" s="9" t="inlineStr"/>
@@ -10116,10 +10428,14 @@
           <t>Spencer Johnson</t>
         </is>
       </c>
-      <c r="D80" s="9" t="inlineStr"/>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F80" s="9" t="inlineStr"/>
@@ -10143,10 +10459,14 @@
           <t>García Márquez Gabriel</t>
         </is>
       </c>
-      <c r="D81" s="9" t="inlineStr"/>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F81" s="9" t="inlineStr"/>
@@ -10170,10 +10490,14 @@
           <t>Gabriel Garcia Marquez</t>
         </is>
       </c>
-      <c r="D82" s="9" t="inlineStr"/>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F82" s="9" t="inlineStr"/>
@@ -10197,10 +10521,14 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="D83" s="9" t="inlineStr"/>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F83" s="9" t="inlineStr"/>
@@ -10224,10 +10552,14 @@
           <t>Graciela Cabal</t>
         </is>
       </c>
-      <c r="D84" s="9" t="inlineStr"/>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F84" s="9" t="inlineStr"/>
@@ -10251,10 +10583,14 @@
           <t>Pablo Neruda</t>
         </is>
       </c>
-      <c r="D85" s="9" t="inlineStr"/>
+      <c r="D85" s="9" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>ACEPTADO</t>
         </is>
       </c>
       <c r="F85" s="9" t="inlineStr"/>

</xml_diff>